<commit_message>
DB brought in new users added models added file to db for accounts pnl for jainam
</commit_message>
<xml_diff>
--- a/jainam/Ayush Keys.xlsx
+++ b/jainam/Ayush Keys.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="66">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -203,6 +203,21 @@
   </si>
   <si>
     <t xml:space="preserve">Hsik733#vS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LD_JAINAM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CL127</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sm@123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">443d71f297e180cae88860</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Xjbo528#kK</t>
   </si>
 </sst>
 </file>
@@ -367,7 +382,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -404,19 +419,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -686,10 +697,20 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:M1048576"/>
-  <sheetFormatPr defaultColWidth="8.859375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="10.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="17.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="11.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="10.48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="25.77"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="15.62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="84.91"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="6.02"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="21.6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="8.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="7.27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="11.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="5.19"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -915,31 +936,31 @@
       <c r="B7" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="C7" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="D7" s="0" t="s">
+      <c r="D7" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="E7" s="0" t="s">
+      <c r="E7" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="F7" s="11" t="s">
+      <c r="F7" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="G7" s="0" t="s">
+      <c r="G7" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="H7" s="0" t="n">
+      <c r="H7" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="I7" s="0" t="s">
+      <c r="I7" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="J7" s="0" t="s">
+      <c r="J7" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="M7" s="0" t="n">
+      <c r="M7" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -947,34 +968,34 @@
       <c r="A8" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="B8" s="12" t="s">
+      <c r="B8" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="C8" s="0" t="s">
+      <c r="C8" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="D8" s="0" t="s">
+      <c r="D8" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="E8" s="0" t="s">
+      <c r="E8" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="F8" s="11" t="s">
+      <c r="F8" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="G8" s="0" t="s">
+      <c r="G8" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="H8" s="0" t="n">
+      <c r="H8" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="I8" s="0" t="s">
+      <c r="I8" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="J8" s="0" t="s">
+      <c r="J8" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="M8" s="0" t="n">
+      <c r="M8" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -994,22 +1015,57 @@
       <c r="E9" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="F9" s="11" t="s">
+      <c r="F9" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="G9" s="0" t="s">
+      <c r="G9" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="H9" s="0" t="n">
+      <c r="H9" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="I9" s="0" t="s">
+      <c r="I9" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="J9" s="0" t="s">
+      <c r="J9" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="M9" s="0" t="n">
+      <c r="M9" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="D10" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="E10" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="F10" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="G10" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="H10" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="J10" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="M10" s="0" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1028,17 +1084,17 @@
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C17" s="3"/>
       <c r="E17" s="8"/>
-      <c r="F17" s="13"/>
+      <c r="F17" s="12"/>
       <c r="G17" s="8"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="14"/>
+      <c r="B18" s="13"/>
       <c r="E18" s="8"/>
       <c r="F18" s="8"/>
       <c r="G18" s="8"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="15"/>
+      <c r="B19" s="14"/>
       <c r="F19" s="8"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1055,6 +1111,7 @@
     <hyperlink ref="C3" r:id="rId2" display="Ram@345"/>
     <hyperlink ref="C6" r:id="rId3" display="Am@234"/>
     <hyperlink ref="C7" r:id="rId4" display="Am@234"/>
+    <hyperlink ref="C10" r:id="rId5" display="Sm@123"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>